<commit_message>
feat: playing around with fit to get the values and fit right, did this by reducing parameter space for fit
</commit_message>
<xml_diff>
--- a/code/data/2025/09/24 - KC Normal Mode Spectroscopy 2-1/goodAtomSelectorFiles/24_09_25_KC_Spectroscopy_2_1_pi_75_375_MHz_100_points_3_atomParameters.xlsx
+++ b/code/data/2025/09/24 - KC Normal Mode Spectroscopy 2-1/goodAtomSelectorFiles/24_09_25_KC_Spectroscopy_2_1_pi_75_375_MHz_100_points_3_atomParameters.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="atomParameters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="goodAtoms" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="goodAtomsConds" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="goodAtomsDic" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="goodAtomsDic" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="goodAtoms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="gootAtomsConds" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,13 +453,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>5.253877343231579</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>1.232193530770019</v>
+        <v>0.8445613971562125</v>
       </c>
       <c r="D2" t="n">
-        <v>6.486070874001598</v>
+        <v>3.844561397156212</v>
       </c>
     </row>
     <row r="3">
@@ -551,13 +551,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>52.71244653989561</v>
+        <v>53</v>
       </c>
       <c r="C9" t="n">
-        <v>1.107183985819574</v>
+        <v>0.1675077680847608</v>
       </c>
       <c r="D9" t="n">
-        <v>53.81963052571518</v>
+        <v>53.16750776808476</v>
       </c>
     </row>
     <row r="10">
@@ -635,13 +635,13 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>57.98562072956702</v>
+        <v>55</v>
       </c>
       <c r="C15" t="n">
-        <v>0.882151608413551</v>
+        <v>0.1567800133780111</v>
       </c>
       <c r="D15" t="n">
-        <v>58.86777233798057</v>
+        <v>55.15678001337801</v>
       </c>
     </row>
     <row r="16">
@@ -663,13 +663,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>15.800225986226</v>
+        <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>1.407212939870078</v>
+        <v>1.097452038055053</v>
       </c>
       <c r="D17" t="n">
-        <v>17.20743892609607</v>
+        <v>13.09745203805505</v>
       </c>
     </row>
     <row r="18">
@@ -691,13 +691,13 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>47.43927198898746</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>1.132186769304099</v>
+        <v>0.6984547469182871</v>
       </c>
       <c r="D19" t="n">
-        <v>48.57145875829156</v>
+        <v>43.69845474691829</v>
       </c>
     </row>
     <row r="20">
@@ -705,13 +705,13 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>21.07340031393687</v>
+        <v>16</v>
       </c>
       <c r="C20" t="n">
-        <v>1.157183895789785</v>
+        <v>0.9353244863159489</v>
       </c>
       <c r="D20" t="n">
-        <v>22.23058420972666</v>
+        <v>16.93532448631595</v>
       </c>
     </row>
     <row r="21">
@@ -733,13 +733,13 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>15.80022597886273</v>
+        <v>11</v>
       </c>
       <c r="C22" t="n">
-        <v>1.482222923921654</v>
+        <v>0.5131841731781606</v>
       </c>
       <c r="D22" t="n">
-        <v>17.28244890278438</v>
+        <v>11.51318417317816</v>
       </c>
     </row>
     <row r="23">
@@ -761,13 +761,13 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>36.892923322157</v>
+        <v>32</v>
       </c>
       <c r="C24" t="n">
-        <v>0.607122108223848</v>
+        <v>0.03917573465150781</v>
       </c>
       <c r="D24" t="n">
-        <v>37.50004543038085</v>
+        <v>32.03917573465151</v>
       </c>
     </row>
     <row r="25">
@@ -803,13 +803,13 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>10.52705165083171</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
-        <v>1.507229235372506</v>
+        <v>1.347688806417864</v>
       </c>
       <c r="D27" t="n">
-        <v>12.03428088620421</v>
+        <v>9.347688806417864</v>
       </c>
     </row>
     <row r="28">
@@ -831,13 +831,13 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>42.16609769899515</v>
+        <v>38</v>
       </c>
       <c r="C29" t="n">
-        <v>0.9071485408640001</v>
+        <v>0.1218496171932202</v>
       </c>
       <c r="D29" t="n">
-        <v>43.07324623985915</v>
+        <v>38.12184961719322</v>
       </c>
     </row>
     <row r="30">
@@ -873,13 +873,13 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>110.7173640983528</v>
+        <v>107</v>
       </c>
       <c r="C32" t="n">
-        <v>1.132180373446317</v>
+        <v>0.8571603118616622</v>
       </c>
       <c r="D32" t="n">
-        <v>111.8495444717992</v>
+        <v>107.8571603118617</v>
       </c>
     </row>
     <row r="33">
@@ -932,10 +932,10 @@
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>0.7071322208212223</v>
+        <v>-0.183709017757792</v>
       </c>
       <c r="D36" t="n">
-        <v>0.7071322208212223</v>
+        <v>-0.183709017757792</v>
       </c>
     </row>
   </sheetData>
@@ -944,6 +944,131 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="J1" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="K1" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="L1" s="1" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.8445613971562125</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1675077680847608</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1567800133780111</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.097452038055053</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.6984547469182871</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9353244863159489</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.5131841731781606</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.03917573465150781</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1.347688806417864</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.1218496171932202</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.8571603118616622</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3.844561397156212</v>
+      </c>
+      <c r="C3" t="n">
+        <v>53.16750776808476</v>
+      </c>
+      <c r="D3" t="n">
+        <v>55.15678001337801</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13.09745203805505</v>
+      </c>
+      <c r="F3" t="n">
+        <v>43.69845474691829</v>
+      </c>
+      <c r="G3" t="n">
+        <v>16.93532448631595</v>
+      </c>
+      <c r="H3" t="n">
+        <v>11.51318417317816</v>
+      </c>
+      <c r="I3" t="n">
+        <v>32.03917573465151</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9.347688806417864</v>
+      </c>
+      <c r="K3" t="n">
+        <v>38.12184961719322</v>
+      </c>
+      <c r="L3" t="n">
+        <v>107.8571603118617</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -974,13 +1099,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>5.253877343231579</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>1.232193530770019</v>
+        <v>0.8445613971562125</v>
       </c>
       <c r="D2" t="n">
-        <v>6.486070874001598</v>
+        <v>3.844561397156212</v>
       </c>
     </row>
     <row r="3">
@@ -988,13 +1113,13 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>52.71244653989561</v>
+        <v>53</v>
       </c>
       <c r="C3" t="n">
-        <v>1.107183985819574</v>
+        <v>0.1675077680847608</v>
       </c>
       <c r="D3" t="n">
-        <v>53.81963052571518</v>
+        <v>53.16750776808476</v>
       </c>
     </row>
     <row r="4">
@@ -1002,13 +1127,13 @@
         <v>13</v>
       </c>
       <c r="B4" t="n">
-        <v>57.98562072956702</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>0.882151608413551</v>
+        <v>0.1567800133780111</v>
       </c>
       <c r="D4" t="n">
-        <v>58.86777233798057</v>
+        <v>55.15678001337801</v>
       </c>
     </row>
     <row r="5">
@@ -1016,13 +1141,13 @@
         <v>15</v>
       </c>
       <c r="B5" t="n">
-        <v>15.800225986226</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>1.407212939870078</v>
+        <v>1.097452038055053</v>
       </c>
       <c r="D5" t="n">
-        <v>17.20743892609607</v>
+        <v>13.09745203805505</v>
       </c>
     </row>
     <row r="6">
@@ -1030,13 +1155,13 @@
         <v>17</v>
       </c>
       <c r="B6" t="n">
-        <v>47.43927198898746</v>
+        <v>43</v>
       </c>
       <c r="C6" t="n">
-        <v>1.132186769304099</v>
+        <v>0.6984547469182871</v>
       </c>
       <c r="D6" t="n">
-        <v>48.57145875829156</v>
+        <v>43.69845474691829</v>
       </c>
     </row>
     <row r="7">
@@ -1044,13 +1169,13 @@
         <v>18</v>
       </c>
       <c r="B7" t="n">
-        <v>21.07340031393687</v>
+        <v>16</v>
       </c>
       <c r="C7" t="n">
-        <v>1.157183895789785</v>
+        <v>0.9353244863159489</v>
       </c>
       <c r="D7" t="n">
-        <v>22.23058420972666</v>
+        <v>16.93532448631595</v>
       </c>
     </row>
     <row r="8">
@@ -1058,13 +1183,13 @@
         <v>20</v>
       </c>
       <c r="B8" t="n">
-        <v>15.80022597886273</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1.482222923921654</v>
+        <v>0.5131841731781606</v>
       </c>
       <c r="D8" t="n">
-        <v>17.28244890278438</v>
+        <v>11.51318417317816</v>
       </c>
     </row>
     <row r="9">
@@ -1072,13 +1197,13 @@
         <v>22</v>
       </c>
       <c r="B9" t="n">
-        <v>36.892923322157</v>
+        <v>32</v>
       </c>
       <c r="C9" t="n">
-        <v>0.607122108223848</v>
+        <v>0.03917573465150781</v>
       </c>
       <c r="D9" t="n">
-        <v>37.50004543038085</v>
+        <v>32.03917573465151</v>
       </c>
     </row>
     <row r="10">
@@ -1086,13 +1211,13 @@
         <v>25</v>
       </c>
       <c r="B10" t="n">
-        <v>10.52705165083171</v>
+        <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>1.507229235372506</v>
+        <v>1.347688806417864</v>
       </c>
       <c r="D10" t="n">
-        <v>12.03428088620421</v>
+        <v>9.347688806417864</v>
       </c>
     </row>
     <row r="11">
@@ -1100,13 +1225,13 @@
         <v>27</v>
       </c>
       <c r="B11" t="n">
-        <v>42.16609769899515</v>
+        <v>38</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9071485408640001</v>
+        <v>0.1218496171932202</v>
       </c>
       <c r="D11" t="n">
-        <v>43.07324623985915</v>
+        <v>38.12184961719322</v>
       </c>
     </row>
     <row r="12">
@@ -1114,13 +1239,13 @@
         <v>30</v>
       </c>
       <c r="B12" t="n">
-        <v>110.7173640983528</v>
+        <v>107</v>
       </c>
       <c r="C12" t="n">
-        <v>1.132180373446317</v>
+        <v>0.8571603118616622</v>
       </c>
       <c r="D12" t="n">
-        <v>111.8495444717992</v>
+        <v>107.8571603118617</v>
       </c>
     </row>
   </sheetData>
@@ -1128,7 +1253,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1165,129 +1290,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="E1" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="F1" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="G1" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="H1" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="J1" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="K1" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="L1" s="1" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="n">
-        <v>1.232193530770019</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1.107183985819574</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.882151608413551</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.407212939870078</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.132186769304099</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1.157183895789785</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.482222923921654</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.607122108223848</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1.507229235372506</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.9071485408640001</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1.132180373446317</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>6.486070874001598</v>
-      </c>
-      <c r="C3" t="n">
-        <v>53.81963052571518</v>
-      </c>
-      <c r="D3" t="n">
-        <v>58.86777233798057</v>
-      </c>
-      <c r="E3" t="n">
-        <v>17.20743892609607</v>
-      </c>
-      <c r="F3" t="n">
-        <v>48.57145875829156</v>
-      </c>
-      <c r="G3" t="n">
-        <v>22.23058420972666</v>
-      </c>
-      <c r="H3" t="n">
-        <v>17.28244890278438</v>
-      </c>
-      <c r="I3" t="n">
-        <v>37.50004543038085</v>
-      </c>
-      <c r="J3" t="n">
-        <v>12.03428088620421</v>
-      </c>
-      <c r="K3" t="n">
-        <v>43.07324623985915</v>
-      </c>
-      <c r="L3" t="n">
-        <v>111.8495444717992</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>